<commit_message>
Avance: Minería de datos
Creé la práctica 4, en documento y video para los compañeros.
</commit_message>
<xml_diff>
--- a/Minería de datos/Practica 3/Análisis de árbol.xlsx
+++ b/Minería de datos/Practica 3/Análisis de árbol.xlsx
@@ -1,39 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositories\Semestre-EneJun2026\Minería de datos\Practica 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Repositorios\Semestre-EneJun2026\Minería de datos\Practica 3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53E9A8F-5A8E-41CB-86CB-FCA1274F8A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BCDBC9-8655-4FAD-8E8D-2A641E38779A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{7E287BC9-8D66-4019-BF8D-4B9C472C75F6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12216" xr2:uid="{7E287BC9-8D66-4019-BF8D-4B9C472C75F6}"/>
   </bookViews>
   <sheets>
     <sheet name="eve" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="53">
   <si>
     <t>Make</t>
   </si>
@@ -1063,18 +1050,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6514CEE5-6049-4212-B845-2550C6118765}">
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:U101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="3" max="3" width="25.88671875" customWidth="1"/>
     <col min="5" max="5" width="11.5546875" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1085,7 +1073,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1096,7 +1084,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1116,7 +1104,7 @@
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1127,7 +1115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1145,8 +1133,14 @@
       <c r="M5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1170,8 +1164,18 @@
         <v>42</v>
       </c>
       <c r="P6" s="1"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R6" s="1"/>
+      <c r="S6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1189,19 +1193,33 @@
         <v>30</v>
       </c>
       <c r="L7" s="1">
-        <f>K7 /$K$16</f>
-        <v>30</v>
+        <f>K7 /$K$19</f>
+        <v>0.3125</v>
       </c>
       <c r="M7" s="2">
         <f>-LOG10(L7) * L7</f>
-        <v>-44.313637641589871</v>
+        <v>0.1578593682249706</v>
       </c>
       <c r="O7" s="1">
         <v>0.85066438927136601</v>
       </c>
       <c r="P7" s="1"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S7" s="1">
+        <v>6</v>
+      </c>
+      <c r="T7" s="1">
+        <f>S7 /$S$16</f>
+        <v>0.31578947368421051</v>
+      </c>
+      <c r="U7" s="2">
+        <f>-LOG10(T7) * T7</f>
+        <v>0.15808495281132168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1226,8 +1244,22 @@
         <f t="shared" ref="M8:M15" si="1">-LOG10(L8) * L8</f>
         <v>-14.481263579988877</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S8" s="1">
+        <v>3</v>
+      </c>
+      <c r="T8" s="1">
+        <f t="shared" ref="T8:T15" si="2">S8 /$S$16</f>
+        <v>0.15789473684210525</v>
+      </c>
+      <c r="U8" s="2">
+        <f t="shared" ref="U8:U16" si="3">-LOG10(T8) * T8</f>
+        <v>0.12657352835260524</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1255,8 +1287,22 @@
         <f t="shared" si="1"/>
         <v>-2.4082399653118496</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="S9" s="1">
+        <v>2</v>
+      </c>
+      <c r="T9" s="1">
+        <f t="shared" si="2"/>
+        <v>0.10526315789473684</v>
+      </c>
+      <c r="U9" s="2">
+        <f t="shared" si="3"/>
+        <v>0.10291827424093135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1284,8 +1330,22 @@
         <f t="shared" si="1"/>
         <v>-2.4082399653118496</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S10" s="1">
+        <v>1</v>
+      </c>
+      <c r="T10" s="1">
+        <f t="shared" si="2"/>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="U10" s="2">
+        <f t="shared" si="3"/>
+        <v>6.7302821102780477E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1313,8 +1373,22 @@
         <f t="shared" si="1"/>
         <v>-4.6689075023018614</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S11" s="1">
+        <v>3</v>
+      </c>
+      <c r="T11" s="1">
+        <f t="shared" si="2"/>
+        <v>0.15789473684210525</v>
+      </c>
+      <c r="U11" s="2">
+        <f t="shared" si="3"/>
+        <v>0.12657352835260524</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1342,8 +1416,22 @@
         <f t="shared" si="1"/>
         <v>-3.4948500216800942</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="S12" s="1">
+        <v>1</v>
+      </c>
+      <c r="T12" s="1">
+        <f t="shared" si="2"/>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="U12" s="2">
+        <f t="shared" si="3"/>
+        <v>6.7302821102780477E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -1371,8 +1459,22 @@
         <f t="shared" si="1"/>
         <v>-0.6020599913279624</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S13" s="1">
+        <v>1</v>
+      </c>
+      <c r="T13" s="1">
+        <f t="shared" si="2"/>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="U13" s="2">
+        <f t="shared" si="3"/>
+        <v>6.7302821102780477E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1400,8 +1502,22 @@
         <f t="shared" si="1"/>
         <v>-14.481263579988877</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="1">
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f t="shared" si="2"/>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="U14" s="2">
+        <f t="shared" si="3"/>
+        <v>6.7302821102780477E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -1426,8 +1542,22 @@
         <f t="shared" si="1"/>
         <v>-19.265919722494797</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S15" s="1">
+        <v>1</v>
+      </c>
+      <c r="T15" s="1">
+        <f t="shared" si="2"/>
+        <v>5.2631578947368418E-2</v>
+      </c>
+      <c r="U15" s="2">
+        <f t="shared" si="3"/>
+        <v>6.7302821102780477E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -1445,12 +1575,16 @@
         <v>1</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" ref="L16" si="2">K16 /$K$16</f>
+        <f t="shared" ref="L16" si="4">K16 /$K$16</f>
         <v>1</v>
       </c>
       <c r="M16" s="2">
-        <f t="shared" ref="M16" si="3">-LOG10(L16) * L16</f>
+        <f t="shared" ref="M16" si="5">-LOG10(L16) * L16</f>
         <v>0</v>
+      </c>
+      <c r="S16">
+        <f>SUM(S7:S15)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
@@ -1467,7 +1601,7 @@
         <v>51</v>
       </c>
       <c r="K17" s="1">
-        <f t="shared" ref="K17:K18" si="4">COUNTIF(A12:A111, "CADILLAC")</f>
+        <f t="shared" ref="K17:K18" si="6">COUNTIF(A12:A111, "CADILLAC")</f>
         <v>1</v>
       </c>
     </row>
@@ -1485,7 +1619,7 @@
         <v>52</v>
       </c>
       <c r="K18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -2441,5 +2575,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>